<commit_message>
Condense row notes, publish to Drive, link deliverables
Moves the shared "egress blocked" explanation out of every row's Notes and
into the README, leaving per-row notes carrying only row-specific facts.
Rebuilds the two-tab workbook from the updated data.

Publishes the Master List as a Google Sheet and the README as a Google Doc,
alongside a 30-folder asset scaffold mirroring the naming convention. A
single two-tab sheet was not possible: this session has Drive file-creation
only and no Sheets API, so tabs cannot be added to an existing spreadsheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XqSsJCBCj3XvoR3Zp97Toe
</commit_message>
<xml_diff>
--- a/out/Logo Library - Research Index.xlsx
+++ b/out/Logo Library - Research Index.xlsx
@@ -1450,12 +1450,12 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>Bank uses a lockup with wave symbol + wordmark; wordmark is the recognised public mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K2" s="8" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="N2" s="6" t="inlineStr">
         <is>
-          <t>State-owned (KBMI 4). Asset not sourced - egress blocked this session; verify against OJK/BI registry and pull official asset.</t>
+          <t>State-owned (KBMI 4).</t>
         </is>
       </c>
     </row>
@@ -1510,12 +1510,12 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Traditional bank with no separate compact symbol in common use</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K3" s="8" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>State-owned (KBMI 4). Asset not sourced - egress blocked this session; verify against OJK/BI registry.</t>
+          <t>State-owned (KBMI 4). Verify: OJK/BI register.</t>
         </is>
       </c>
     </row>
@@ -1570,12 +1570,12 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>BNI "46" mark is widely used standalone in compact checkout UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>State-owned (KBMI 4). Asset not sourced - egress blocked this session; verify against OJK/BI registry.</t>
+          <t>State-owned (KBMI 4). Verify: OJK/BI register.</t>
         </is>
       </c>
     </row>
@@ -1630,12 +1630,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>BCA has a distinct symbol used standalone on Indonesian checkout screens</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K5" s="8" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>Largest private bank. Asset not sourced - egress blocked this session; verify against OJK/BI registry.</t>
+          <t>Largest private bank. Verify: OJK/BI register.</t>
         </is>
       </c>
     </row>
@@ -1690,12 +1690,12 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>No separate compact symbol commonly used</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>State-owned. Asset not sourced - egress blocked this session; verify against OJK/BI registry.</t>
+          <t>State-owned. Verify: OJK/BI register.</t>
         </is>
       </c>
     </row>
@@ -1750,12 +1750,12 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Post-2021 merger identity; wordmark+symbol lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K7" s="8" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>Formed 2021 from BRIsyariah/BNI Syariah/Mandiri Syariah merger. Asset not sourced - egress blocked.</t>
+          <t>Formed 2021 from BRIsyariah/BNI Syariah/Mandiri Syariah merger.</t>
         </is>
       </c>
     </row>
@@ -1810,12 +1810,12 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark with local suffix; no standalone compact symbol</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>Asset not sourced - egress blocked this session; verify against OJK/BI registry.</t>
+          <t>Verify: OJK/BI register.</t>
         </is>
       </c>
     </row>
@@ -1870,12 +1870,12 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the recognised mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K9" s="8" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>MUFG-controlled. Asset not sourced - egress blocked this session.</t>
+          <t>MUFG-controlled.</t>
         </is>
       </c>
     </row>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the public mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>Owned by Bangkok Bank. Asset not sourced - egress blocked this session.</t>
+          <t>Owned by Bangkok Bank.</t>
         </is>
       </c>
     </row>
@@ -1990,12 +1990,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Traditional bank wordmark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>Asset not sourced - egress blocked this session; verify against OJK/BI registry.</t>
+          <t>Verify: OJK/BI register.</t>
         </is>
       </c>
     </row>
@@ -2050,12 +2050,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark; dropped "NISP" in 2023 rebrand</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>Rebranded from OCBC NISP (2023) - do not use pre-rebrand asset. Egress blocked this session.</t>
+          <t>Rebranded from OCBC NISP (2023) - do not use pre-rebrand asset.</t>
         </is>
       </c>
     </row>
@@ -2110,12 +2110,12 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Group tiger-head + wordmark lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>Asset not sourced - egress blocked this session.</t>
+          <t>Candidate row; regulator check and asset sourcing outstanding.</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2166,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Group SMBC wordmark post-rebrand</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>Renamed from Bank BTPN effective 2 Oct 2024 - do NOT use BTPN asset. Official domain changed post-rebrand; confirm before sourcing. Egress blocked this session.</t>
+          <t>Renamed from Bank BTPN effective 2 Oct 2024 - do NOT use BTPN asset. Official domain changed post-rebrand; confirm before sourcing.</t>
         </is>
       </c>
     </row>
@@ -2226,12 +2226,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Wordmark with symbol lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>CT Corp group. Asset not sourced - egress blocked this session.</t>
+          <t>CT Corp group.</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2286,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>KB group wordmark post-rebrand</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>Rebranded from KB Bukopin (2024) - confirm current name/domain. Egress blocked this session.</t>
+          <t>Rebranded from KB Bukopin (2024) - confirm current name/domain.</t>
         </is>
       </c>
     </row>
@@ -2346,12 +2346,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>Retains BTPN Syariah name despite parent rebrand - confirm. Egress blocked this session.</t>
+          <t>Retains BTPN Syariah name despite parent rebrand - confirm.</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>Asset not sourced - egress blocked this session.</t>
+          <t>Candidate row; regulator check and asset sourcing outstanding.</t>
         </is>
       </c>
     </row>
@@ -2466,12 +2466,12 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Regional development bank wordmark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K19" s="8" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>Regional (BPD West Java). Asset not sourced - egress blocked this session.</t>
+          <t>Regional (BPD West Java).</t>
         </is>
       </c>
     </row>
@@ -2526,12 +2526,12 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Regional development bank wordmark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>Regional (Jakarta). Asset not sourced - egress blocked this session.</t>
+          <t>Regional (Jakarta).</t>
         </is>
       </c>
     </row>
@@ -2586,12 +2586,12 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Regional development bank wordmark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>Regional (East Java). Asset not sourced - egress blocked this session.</t>
+          <t>Regional (East Java).</t>
         </is>
       </c>
     </row>
@@ -2646,12 +2646,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>First Indonesian sharia bank. Asset not sourced - egress blocked this session.</t>
+          <t>First Indonesian sharia bank.</t>
         </is>
       </c>
     </row>
@@ -2706,12 +2706,12 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Digital-first bank; app icon is the most recognised public mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>Digital bank. Asset not sourced - egress blocked this session.</t>
+          <t>Digital bank.</t>
         </is>
       </c>
     </row>
@@ -2766,12 +2766,12 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Digital bank; app icon dominates consumer recognition</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>Sea Group. Asset not sourced - egress blocked this session.</t>
+          <t>Sea Group.</t>
         </is>
       </c>
     </row>
@@ -2826,12 +2826,12 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Digital bank; app icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K25" s="8" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>CT Corp group. Asset not sourced - egress blocked this session.</t>
+          <t>CT Corp group.</t>
         </is>
       </c>
     </row>
@@ -2886,12 +2886,12 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Digital bank; app icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K26" s="8" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>Grab/Singtel/Emtek backed. Asset not sourced - egress blocked this session.</t>
+          <t>Grab/Singtel/Emtek backed.</t>
         </is>
       </c>
     </row>
@@ -2946,12 +2946,12 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Digital bank; app icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K27" s="8" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>Asset not sourced - egress blocked this session.</t>
+          <t>Candidate row; regulator check and asset sourcing outstanding.</t>
         </is>
       </c>
     </row>
@@ -3006,12 +3006,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Digital sub-brand; app icon is the recognised mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>Distinct brand from BCA parent - keep separate row. Egress blocked this session.</t>
+          <t>Distinct brand from BCA parent - keep separate row.</t>
         </is>
       </c>
     </row>
@@ -3066,12 +3066,12 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>HSBC hexagon symbol is used standalone in compact UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>Local arm of global group. Asset not sourced - egress blocked this session.</t>
+          <t>Local arm of global group.</t>
         </is>
       </c>
     </row>
@@ -3126,12 +3126,12 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K30" s="8" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>Acquired Citi Indonesia consumer business (2023). Egress blocked this session.</t>
+          <t>Acquired Citi Indonesia consumer business (2023).</t>
         </is>
       </c>
     </row>
@@ -3186,12 +3186,12 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Citi wordmark with arc is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr">
@@ -3246,12 +3246,12 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>E-wallet whose rounded-square app icon is its most recognised public mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>Top-5 wallet (GoTo group). Asset not sourced - egress blocked this session; verify against BI e-money licence list.</t>
+          <t>Top-5 wallet (GoTo group). Verify: BI e-money licence list.</t>
         </is>
       </c>
     </row>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Purple app icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>Top-5 wallet (Grab-controlled). Asset not sourced - egress blocked this session.</t>
+          <t>Top-5 wallet (Grab-controlled).</t>
         </is>
       </c>
     </row>
@@ -3366,12 +3366,12 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>Top-5 wallet (Ant Group backed). Asset not sourced - egress blocked this session.</t>
+          <t>Top-5 wallet (Ant Group backed).</t>
         </is>
       </c>
     </row>
@@ -3426,12 +3426,12 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>In-app wallet brand; app-icon style mark used at checkout</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K35" s="8" t="inlineStr">
@@ -3486,12 +3486,12 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K36" s="8" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>Top-5 wallet (Telkomsel/state-linked). Asset not sourced - egress blocked this session.</t>
+          <t>Top-5 wallet (Telkomsel/state-linked).</t>
         </is>
       </c>
     </row>
@@ -3546,12 +3546,12 @@
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>App icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J37" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K37" s="8" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>Astra group. Asset not sourced - egress blocked this session.</t>
+          <t>Astra group.</t>
         </is>
       </c>
     </row>
@@ -3606,12 +3606,12 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>App icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K38" s="8" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>Indomaret-affiliated wallet. Confirm current operating status. Egress blocked this session.</t>
+          <t>Indomaret-affiliated wallet. Confirm current operating status.</t>
         </is>
       </c>
     </row>
@@ -3666,12 +3666,12 @@
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>Primarily a PSP brand; wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K39" s="8" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>Payment gateway + wallet. Asset not sourced - egress blocked this session.</t>
+          <t>Payment gateway + wallet.</t>
         </is>
       </c>
     </row>
@@ -3726,12 +3726,12 @@
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>App icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K40" s="8" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>Transfer/remittance app. Asset not sourced - egress blocked this session.</t>
+          <t>Transfer/remittance app.</t>
         </is>
       </c>
     </row>
@@ -3786,12 +3786,12 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>App icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K41" s="8" t="inlineStr">
@@ -3890,12 +3890,12 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>Retail chain identity is a horizontal wordmark used on storefront and checkout</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K43" s="8" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>Market leader. Also now operates acquired Lawson Indonesia stores. Egress blocked this session.</t>
+          <t>Market leader. Also now operates acquired Lawson Indonesia stores.</t>
         </is>
       </c>
     </row>
@@ -3950,12 +3950,12 @@
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>Horizontal wordmark is the storefront and payment-channel mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K44" s="8" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>Market leader. Asset not sourced - egress blocked this session.</t>
+          <t>Market leader.</t>
         </is>
       </c>
     </row>
@@ -4010,12 +4010,12 @@
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>Horizontal wordmark, same family as Alfamart</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K45" s="8" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>Confirm official domain. Asset not sourced - egress blocked this session.</t>
+          <t>Confirm official domain.</t>
         </is>
       </c>
     </row>
@@ -4070,12 +4070,12 @@
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>Circle K roundel is used standalone and reads well compact</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K46" s="8" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>Confirm current franchise status in Indonesia. Egress blocked this session.</t>
+          <t>Confirm current franchise status in Indonesia.</t>
         </is>
       </c>
     </row>
@@ -4130,12 +4130,12 @@
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>Milk-can roundel is the recognised standalone mark</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K47" s="8" t="inlineStr">
@@ -4190,12 +4190,12 @@
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>Wordmark with green/blue stripes is the standard storefront mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K48" s="8" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="N48" s="6" t="inlineStr">
         <is>
-          <t>Confirm current footprint in Indonesia. Egress blocked this session.</t>
+          <t>Confirm current footprint in Indonesia.</t>
         </is>
       </c>
     </row>
@@ -4330,12 +4330,12 @@
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>Orange bag app icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K51" s="8" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="N51" s="6" t="inlineStr">
         <is>
-          <t>Market leader. Asset not sourced - egress blocked this session.</t>
+          <t>Market leader.</t>
         </is>
       </c>
     </row>
@@ -4390,12 +4390,12 @@
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>Green owl app icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K52" s="8" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>TikTok acquired majority stake (2024); brand still operates. Egress blocked this session.</t>
+          <t>TikTok acquired majority stake (2024); brand still operates.</t>
         </is>
       </c>
     </row>
@@ -4450,12 +4450,12 @@
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K53" s="8" t="inlineStr">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>Alibaba group. Asset not sourced - egress blocked this session.</t>
+          <t>Alibaba group.</t>
         </is>
       </c>
     </row>
@@ -4510,12 +4510,12 @@
       </c>
       <c r="I54" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K54" s="8" t="inlineStr">
@@ -4570,12 +4570,12 @@
       </c>
       <c r="I55" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K55" s="8" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>Djarum/GDP Venture group. Asset not sourced - egress blocked this session.</t>
+          <t>Djarum/GDP Venture group.</t>
         </is>
       </c>
     </row>
@@ -4630,12 +4630,12 @@
       </c>
       <c r="I56" s="6" t="inlineStr">
         <is>
-          <t>Fashion brand uses a horizontal wordmark as primary mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K56" s="8" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>Asset not sourced - egress blocked this session.</t>
+          <t>Candidate row; regulator check and asset sourcing outstanding.</t>
         </is>
       </c>
     </row>
@@ -4690,12 +4690,12 @@
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>Note mark is the recognised compact brand</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K57" s="8" t="inlineStr">
@@ -4750,12 +4750,12 @@
       </c>
       <c r="I58" s="6" t="inlineStr">
         <is>
-          <t>App icon is the primary consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K58" s="8" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="N58" s="6" t="inlineStr">
         <is>
-          <t>Primarily BNPL/paylater rather than pure marketplace - confirm category fit. Egress blocked this session.</t>
+          <t>Primarily BNPL/paylater rather than pure marketplace - confirm category fit.</t>
         </is>
       </c>
     </row>
@@ -4810,12 +4810,12 @@
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the primary brand mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J59" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K59" s="8" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="N59" s="6" t="inlineStr">
         <is>
-          <t>Mother/baby vertical (Sirclo group). Confirm current status. Egress blocked this session.</t>
+          <t>Mother/baby vertical (Sirclo group). Confirm current status.</t>
         </is>
       </c>
     </row>
@@ -4870,12 +4870,12 @@
       </c>
       <c r="I60" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the primary brand mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K60" s="8" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="N60" s="6" t="inlineStr">
         <is>
-          <t>Beauty vertical. Asset not sourced - egress blocked this session.</t>
+          <t>Beauty vertical.</t>
         </is>
       </c>
     </row>
@@ -5014,12 +5014,12 @@
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>Red "DBS" wordmark is the standard mark; no separate symbol in common compact use</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K63" s="8" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="N63" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS licensed-banks register. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: MAS register.</t>
         </is>
       </c>
     </row>
@@ -5078,12 +5078,12 @@
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K64" s="8" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS register. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: MAS register.</t>
         </is>
       </c>
     </row>
@@ -5142,12 +5142,12 @@
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J65" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K65" s="8" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="N65" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS register. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: MAS register.</t>
         </is>
       </c>
     </row>
@@ -5206,12 +5206,12 @@
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark with twist symbol</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J66" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K66" s="8" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS register. Consider whether local variants duplicate the international row.</t>
+          <t>Verify: MAS register. Consider whether local variants duplicate the international row.</t>
         </is>
       </c>
     </row>
@@ -5270,12 +5270,12 @@
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>Citi wordmark with arc</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J67" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K67" s="8" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS register. Consider whether local variants duplicate the international row.</t>
+          <t>Verify: MAS register. Consider whether local variants duplicate the international row.</t>
         </is>
       </c>
     </row>
@@ -5334,12 +5334,12 @@
       </c>
       <c r="I68" s="6" t="inlineStr">
         <is>
-          <t>Group tiger-head + wordmark lockup</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J68" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K68" s="8" t="inlineStr">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="N68" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS register. Same group mark as Maybank MY - confirm whether a distinct SG asset is needed.</t>
+          <t>Verify: MAS register. Same group mark as Maybank MY - confirm whether a distinct SG asset is needed.</t>
         </is>
       </c>
     </row>
@@ -5398,12 +5398,12 @@
       </c>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>Tiger-head + wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J69" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K69" s="8" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="N69" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM licensed-institutions list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5462,12 +5462,12 @@
       </c>
       <c r="I70" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J70" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K70" s="8" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="N70" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5526,12 +5526,12 @@
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>Traditional bank wordmark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J71" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K71" s="8" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="N71" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5590,12 +5590,12 @@
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J72" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K72" s="8" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="N72" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5654,12 +5654,12 @@
       </c>
       <c r="I73" s="6" t="inlineStr">
         <is>
-          <t>Traditional bank wordmark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J73" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K73" s="8" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="N73" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5718,12 +5718,12 @@
       </c>
       <c r="I74" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J74" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K74" s="8" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5782,12 +5782,12 @@
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K75" s="8" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="N75" s="6" t="inlineStr">
         <is>
-          <t>Verify against BNM list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -5846,12 +5846,12 @@
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>Blue magnolia/leaf symbol is used standalone in Thai checkout UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J76" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K76" s="8" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="N76" s="6" t="inlineStr">
         <is>
-          <t>Verify against Bank of Thailand register. Owns PermataBank Indonesia. Egress blocked this session.</t>
+          <t>Verify: BOT register. Owns PermataBank Indonesia.</t>
         </is>
       </c>
     </row>
@@ -5910,12 +5910,12 @@
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>Green sheaf symbol is used standalone and is highly recognised in Thai UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J77" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K77" s="8" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="N77" s="6" t="inlineStr">
         <is>
-          <t>Verify against BOT register. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BOT register.</t>
         </is>
       </c>
     </row>
@@ -5974,12 +5974,12 @@
       </c>
       <c r="I78" s="6" t="inlineStr">
         <is>
-          <t>Purple shield/leaf symbol is used standalone in Thai UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K78" s="8" t="inlineStr">
@@ -5995,7 +5995,7 @@
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>Verify against BOT register. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BOT register.</t>
         </is>
       </c>
     </row>
@@ -6038,12 +6038,12 @@
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>Blue symbol used standalone in Thai UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K79" s="8" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>Verify against BOT register. State-owned. Egress blocked this session.</t>
+          <t>Verify: BOT register. State-owned.</t>
         </is>
       </c>
     </row>
@@ -6102,12 +6102,12 @@
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>Yellow symbol used standalone in Thai UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J80" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K80" s="8" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>Verify against BOT register. MUFG-controlled. Egress blocked this session.</t>
+          <t>Verify: BOT register. MUFG-controlled.</t>
         </is>
       </c>
     </row>
@@ -6166,12 +6166,12 @@
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>Lowercase "ttb" wordmark is the post-merger mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K81" s="8" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="N81" s="6" t="inlineStr">
         <is>
-          <t>Formed from TMB + Thanachart merger - do NOT use legacy TMB or Thanachart assets. Verify against BOT register.</t>
+          <t>Formed from TMB + Thanachart merger - do NOT use legacy TMB or Thanachart assets. Verify: BOT register.</t>
         </is>
       </c>
     </row>
@@ -6230,12 +6230,12 @@
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J82" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K82" s="8" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="N82" s="6" t="inlineStr">
         <is>
-          <t>Verify against BSP directory. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -6294,12 +6294,12 @@
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J83" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K83" s="8" t="inlineStr">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>Verify against BSP directory. Rebranded identity in recent years - use current asset only.</t>
+          <t>Verify: BSP directory. Rebranded identity in recent years - use current asset only.</t>
         </is>
       </c>
     </row>
@@ -6358,12 +6358,12 @@
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J84" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K84" s="8" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>Verify against BSP directory. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -6422,12 +6422,12 @@
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K85" s="8" t="inlineStr">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="N85" s="6" t="inlineStr">
         <is>
-          <t>State-owned. Verify against BSP directory. Egress blocked this session.</t>
+          <t>State-owned. Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -6486,12 +6486,12 @@
       </c>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K86" s="8" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="N86" s="6" t="inlineStr">
         <is>
-          <t>Verify against BSP directory. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -6550,12 +6550,12 @@
       </c>
       <c r="I87" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K87" s="8" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="N87" s="6" t="inlineStr">
         <is>
-          <t>Verify against BSP directory. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -6614,12 +6614,12 @@
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>Green/gold wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J88" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K88" s="8" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="N88" s="6" t="inlineStr">
         <is>
-          <t>Verify against State Bank of Vietnam list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -6678,12 +6678,12 @@
       </c>
       <c r="I89" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K89" s="8" t="inlineStr">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="N89" s="6" t="inlineStr">
         <is>
-          <t>Verify against SBV list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -6742,12 +6742,12 @@
       </c>
       <c r="I90" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J90" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K90" s="8" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="N90" s="6" t="inlineStr">
         <is>
-          <t>Verify against SBV list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -6806,12 +6806,12 @@
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>Red wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K91" s="8" t="inlineStr">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="N91" s="6" t="inlineStr">
         <is>
-          <t>Verify against SBV list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -6870,12 +6870,12 @@
       </c>
       <c r="I92" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J92" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K92" s="8" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="N92" s="6" t="inlineStr">
         <is>
-          <t>Verify against SBV list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -6934,12 +6934,12 @@
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J93" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K93" s="8" t="inlineStr">
@@ -6955,7 +6955,7 @@
       </c>
       <c r="N93" s="6" t="inlineStr">
         <is>
-          <t>Verify against SBV list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -6998,12 +6998,12 @@
       </c>
       <c r="I94" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J94" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K94" s="8" t="inlineStr">
@@ -7019,7 +7019,7 @@
       </c>
       <c r="N94" s="6" t="inlineStr">
         <is>
-          <t>Verify against SBV list. Asset not sourced - egress blocked this session.</t>
+          <t>Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -7062,12 +7062,12 @@
       </c>
       <c r="I95" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J95" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K95" s="8" t="inlineStr">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="N95" s="6" t="inlineStr">
         <is>
-          <t>Verify against National Bank of Cambodia list. Lower-priority market per brief.</t>
+          <t>Verify: NBC list. Lower-priority market per brief.</t>
         </is>
       </c>
     </row>
@@ -7126,12 +7126,12 @@
       </c>
       <c r="I96" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J96" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K96" s="8" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="N96" s="6" t="inlineStr">
         <is>
-          <t>Verify against Bank of the Lao PDR. Lower-priority market; limited asset availability expected.</t>
+          <t>Verify: BOL list. Lower-priority market; limited asset availability expected.</t>
         </is>
       </c>
     </row>
@@ -7190,12 +7190,12 @@
       </c>
       <c r="I97" s="6" t="inlineStr">
         <is>
-          <t>Wordmark lockup is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J97" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K97" s="8" t="inlineStr">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="N97" s="6" t="inlineStr">
         <is>
-          <t>Verify against Brunei Darussalam Central Bank. Lower-priority market per brief.</t>
+          <t>Verify: BDCB list. Lower-priority market per brief.</t>
         </is>
       </c>
     </row>
@@ -7298,12 +7298,12 @@
       </c>
       <c r="I99" s="6" t="inlineStr">
         <is>
-          <t>Grab green app-icon style mark is the recognised wallet brand</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K99" s="8" t="inlineStr">
@@ -7362,12 +7362,12 @@
       </c>
       <c r="I100" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K100" s="8" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="N100" s="6" t="inlineStr">
         <is>
-          <t>Verify against MAS e-money/major payment institution register. Egress blocked this session.</t>
+          <t>Verify: MAS register.</t>
         </is>
       </c>
     </row>
@@ -7426,12 +7426,12 @@
       </c>
       <c r="I101" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J101" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K101" s="8" t="inlineStr">
@@ -7490,12 +7490,12 @@
       </c>
       <c r="I102" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J102" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K102" s="8" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="N102" s="6" t="inlineStr">
         <is>
-          <t>Confirm current operating status and ownership (Pine Labs group) before sourcing. Egress blocked this session.</t>
+          <t>Confirm current operating status and ownership (Pine Labs group) before sourcing.</t>
         </is>
       </c>
     </row>
@@ -7554,12 +7554,12 @@
       </c>
       <c r="I103" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J103" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K103" s="8" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="N103" s="6" t="inlineStr">
         <is>
-          <t>Multi-currency card/wallet. Verify against MAS register. Egress blocked this session.</t>
+          <t>Multi-currency card/wallet. Verify: MAS register.</t>
         </is>
       </c>
     </row>
@@ -7618,12 +7618,12 @@
       </c>
       <c r="I104" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark in Malaysia</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J104" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K104" s="8" t="inlineStr">
@@ -7639,7 +7639,7 @@
       </c>
       <c r="N104" s="6" t="inlineStr">
         <is>
-          <t>Market leader MY. Verify against BNM e-money licensee list. Egress blocked this session.</t>
+          <t>Market leader MY. Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -7682,12 +7682,12 @@
       </c>
       <c r="I105" s="6" t="inlineStr">
         <is>
-          <t>Grab app-icon style mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J105" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K105" s="8" t="inlineStr">
@@ -7746,12 +7746,12 @@
       </c>
       <c r="I106" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J106" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K106" s="8" t="inlineStr">
@@ -7767,7 +7767,7 @@
       </c>
       <c r="N106" s="6" t="inlineStr">
         <is>
-          <t>Axiata group. Verify against BNM list. Egress blocked this session.</t>
+          <t>Axiata group. Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -7810,12 +7810,12 @@
       </c>
       <c r="I107" s="6" t="inlineStr">
         <is>
-          <t>In-app wallet brand; app-icon style mark used at checkout</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J107" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K107" s="8" t="inlineStr">
@@ -7874,12 +7874,12 @@
       </c>
       <c r="I108" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J108" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K108" s="8" t="inlineStr">
@@ -7895,7 +7895,7 @@
       </c>
       <c r="N108" s="6" t="inlineStr">
         <is>
-          <t>Capital A/AirAsia group. Verify against BNM list. Egress blocked this session.</t>
+          <t>Capital A/AirAsia group. Verify: BNM list.</t>
         </is>
       </c>
     </row>
@@ -7938,12 +7938,12 @@
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J109" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K109" s="8" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="N109" s="6" t="inlineStr">
         <is>
-          <t>Ascend Money group; operates across SEA incl. Indonesia. Verify against BOT e-money list.</t>
+          <t>Ascend Money group; operates across SEA incl. Indonesia. Verify: BOT register.</t>
         </is>
       </c>
     </row>
@@ -8002,12 +8002,12 @@
       </c>
       <c r="I110" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J110" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K110" s="8" t="inlineStr">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="N110" s="6" t="inlineStr">
         <is>
-          <t>Confirm current branding/ownership arrangement. Verify against BOT list.</t>
+          <t>Confirm current branding/ownership arrangement. Verify: BOT register.</t>
         </is>
       </c>
     </row>
@@ -8066,12 +8066,12 @@
       </c>
       <c r="I111" s="6" t="inlineStr">
         <is>
-          <t>In-app wallet brand; app-icon style mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J111" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K111" s="8" t="inlineStr">
@@ -8130,12 +8130,12 @@
       </c>
       <c r="I112" s="6" t="inlineStr">
         <is>
-          <t>Grab app-icon style mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J112" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K112" s="8" t="inlineStr">
@@ -8194,12 +8194,12 @@
       </c>
       <c r="I113" s="6" t="inlineStr">
         <is>
-          <t>Blue app icon is the dominant consumer mark in the Philippines</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J113" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K113" s="8" t="inlineStr">
@@ -8215,7 +8215,7 @@
       </c>
       <c r="N113" s="6" t="inlineStr">
         <is>
-          <t>Market leader PH. Verify against BSP e-money issuer list. Egress blocked this session.</t>
+          <t>Market leader PH. Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -8258,12 +8258,12 @@
       </c>
       <c r="I114" s="6" t="inlineStr">
         <is>
-          <t>App icon is the dominant consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J114" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K114" s="8" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="N114" s="6" t="inlineStr">
         <is>
-          <t>Rebranded from PayMaya - do NOT use legacy PayMaya asset. Verify against BSP list.</t>
+          <t>Rebranded from PayMaya - do NOT use legacy PayMaya asset. Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -8322,12 +8322,12 @@
       </c>
       <c r="I115" s="6" t="inlineStr">
         <is>
-          <t>Grab app-icon style mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J115" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K115" s="8" t="inlineStr">
@@ -8386,12 +8386,12 @@
       </c>
       <c r="I116" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J116" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K116" s="8" t="inlineStr">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="N116" s="6" t="inlineStr">
         <is>
-          <t>Crypto-adjacent wallet - confirm it fits the intended payment-method grouping. Verify against BSP list.</t>
+          <t>Crypto-adjacent wallet - confirm it fits the intended payment-method grouping. Verify: BSP directory.</t>
         </is>
       </c>
     </row>
@@ -8450,12 +8450,12 @@
       </c>
       <c r="I117" s="6" t="inlineStr">
         <is>
-          <t>Pink app icon is the dominant consumer mark in Vietnam</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J117" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K117" s="8" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="N117" s="6" t="inlineStr">
         <is>
-          <t>Market leader VN. Verify against State Bank of Vietnam licensee list.</t>
+          <t>Market leader VN. Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -8514,12 +8514,12 @@
       </c>
       <c r="I118" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K118" s="8" t="inlineStr">
@@ -8535,7 +8535,7 @@
       </c>
       <c r="N118" s="6" t="inlineStr">
         <is>
-          <t>Rebranded in recent years - use current asset. Verify against SBV list.</t>
+          <t>Rebranded in recent years - use current asset. Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -8578,12 +8578,12 @@
       </c>
       <c r="I119" s="6" t="inlineStr">
         <is>
-          <t>App icon / QR brand mark is the recognised mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K119" s="8" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="N119" s="6" t="inlineStr">
         <is>
-          <t>Primarily a payment gateway/QR scheme - confirm category fit. Verify against SBV list.</t>
+          <t>Primarily a payment gateway/QR scheme - confirm category fit. Verify: SBV list.</t>
         </is>
       </c>
     </row>
@@ -8642,12 +8642,12 @@
       </c>
       <c r="I120" s="6" t="inlineStr">
         <is>
-          <t>In-app wallet brand; app-icon style mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J120" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K120" s="8" t="inlineStr">
@@ -8750,12 +8750,12 @@
       </c>
       <c r="I122" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J122" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K122" s="8" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="N122" s="6" t="inlineStr">
         <is>
-          <t>Verify against National Bank of Cambodia. Lower-priority market per brief.</t>
+          <t>Verify: NBC list. Lower-priority market per brief.</t>
         </is>
       </c>
     </row>
@@ -8858,12 +8858,12 @@
       </c>
       <c r="I124" s="6" t="inlineStr">
         <is>
-          <t>App icon is the recognised consumer mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J124" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K124" s="8" t="inlineStr">
@@ -8918,12 +8918,12 @@
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>Red/white hexagon is a true standalone symbol that reads well in compact UI</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J125" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K125" s="8" t="inlineStr">
@@ -8939,7 +8939,7 @@
       </c>
       <c r="N125" s="6" t="inlineStr">
         <is>
-          <t>Globally recognised; relevant to Indonesian cross-border transfers. Asset not sourced - egress blocked this session.</t>
+          <t>Globally recognised; relevant to Indonesian cross-border transfers.</t>
         </is>
       </c>
     </row>
@@ -8978,12 +8978,12 @@
       </c>
       <c r="I126" s="6" t="inlineStr">
         <is>
-          <t>Citi wordmark with red arc is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J126" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K126" s="8" t="inlineStr">
@@ -8999,7 +8999,7 @@
       </c>
       <c r="N126" s="6" t="inlineStr">
         <is>
-          <t>Globally recognised. Asset not sourced - egress blocked this session.</t>
+          <t>Globally recognised.</t>
         </is>
       </c>
     </row>
@@ -9038,12 +9038,12 @@
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>Group wordmark with twist symbol</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J127" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K127" s="8" t="inlineStr">
@@ -9059,7 +9059,7 @@
       </c>
       <c r="N127" s="6" t="inlineStr">
         <is>
-          <t>Globally recognised. Asset not sourced - egress blocked this session.</t>
+          <t>Globally recognised.</t>
         </is>
       </c>
     </row>
@@ -9098,12 +9098,12 @@
       </c>
       <c r="I128" s="6" t="inlineStr">
         <is>
-          <t>Double-P monogram is a true standalone symbol widely used at checkout</t>
+          <t>Standalone symbol, reads well compact</t>
         </is>
       </c>
       <c r="J128" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square-ish icon)</t>
+          <t>TBD (square-ish)</t>
         </is>
       </c>
       <c r="K128" s="8" t="inlineStr">
@@ -9119,7 +9119,7 @@
       </c>
       <c r="N128" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session (egress blocked) - confirm on PayPal's own site before including.</t>
+          <t>Indonesia support unconfirmed - confirm on PayPal's own site before including.</t>
         </is>
       </c>
     </row>
@@ -9158,12 +9158,12 @@
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>Green flag-style app icon is the recognised compact mark</t>
+          <t>App icon is the most recognised mark</t>
         </is>
       </c>
       <c r="J129" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect square icon)</t>
+          <t>TBD (square)</t>
         </is>
       </c>
       <c r="K129" s="8" t="inlineStr">
@@ -9179,7 +9179,7 @@
       </c>
       <c r="N129" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session - confirm IDR receive support on wise.com before including.</t>
+          <t>Indonesia support unconfirmed - confirm IDR receive support on wise.com before including.</t>
         </is>
       </c>
     </row>
@@ -9218,12 +9218,12 @@
       </c>
       <c r="I130" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J130" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K130" s="8" t="inlineStr">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="N130" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session - confirm on payoneer.com before including.</t>
+          <t>Indonesia support unconfirmed - confirm on payoneer.com before including.</t>
         </is>
       </c>
     </row>
@@ -9278,12 +9278,12 @@
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>Purple wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J131" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K131" s="8" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="N131" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session - Skrill country coverage changes; confirm before including.</t>
+          <t>Indonesia support unconfirmed - Skrill country coverage changes; confirm before including.</t>
         </is>
       </c>
     </row>
@@ -9338,12 +9338,12 @@
       </c>
       <c r="I132" s="6" t="inlineStr">
         <is>
-          <t>Yellow/black wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J132" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K132" s="8" t="inlineStr">
@@ -9398,12 +9398,12 @@
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J133" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K133" s="8" t="inlineStr">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="N133" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session - confirm before including.</t>
+          <t>Indonesia support unconfirmed - confirm before including.</t>
         </is>
       </c>
     </row>
@@ -9458,12 +9458,12 @@
       </c>
       <c r="I134" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J134" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K134" s="8" t="inlineStr">
@@ -9479,7 +9479,7 @@
       </c>
       <c r="N134" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session - confirm before including. Parent group also operates Zepz/Sendwave brands.</t>
+          <t>Indonesia support unconfirmed - confirm before including. Parent group also operates Zepz/Sendwave brands.</t>
         </is>
       </c>
     </row>
@@ -9518,12 +9518,12 @@
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>Wordmark is the standard mark</t>
+          <t>Wordmark is the standard public mark</t>
         </is>
       </c>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>TBD (expect horizontal wordmark)</t>
+          <t>TBD (horizontal)</t>
         </is>
       </c>
       <c r="K135" s="8" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="N135" s="6" t="inlineStr">
         <is>
-          <t>Indonesia support NOT verified this session - confirm before including.</t>
+          <t>Indonesia support unconfirmed - confirm before including.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill missing website URLs on the new international rows
fetch_logos.py's two strongest resolvers (brand-site scraping and the
favicon-service fallback) both return no candidates when a row's website
column is empty - and all 44 non-renamed international rows added for the
Wise/PandaRemit expansion had it blank. Left as-is, the GitHub Actions
fetch run would have skipped the brief's top-priority source for every one
of them and fallen back to app-store search and Wikimedia only.

Fills in the official site for all 44 rows so a fetch run resolves them the
same way as every other row in the sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XqSsJCBCj3XvoR3Zp97Toe
</commit_message>
<xml_diff>
--- a/out/Logo Library - Research Index.xlsx
+++ b/out/Logo Library - Research Index.xlsx
@@ -13329,7 +13329,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F199" s="8" t="inlineStr"/>
+      <c r="F199" s="9" t="inlineStr">
+        <is>
+          <t>https://www.chase.com</t>
+        </is>
+      </c>
       <c r="G199" s="8" t="inlineStr"/>
       <c r="H199" s="8" t="inlineStr">
         <is>
@@ -13389,7 +13393,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F200" s="8" t="inlineStr"/>
+      <c r="F200" s="9" t="inlineStr">
+        <is>
+          <t>https://www.bankofamerica.com</t>
+        </is>
+      </c>
       <c r="G200" s="8" t="inlineStr"/>
       <c r="H200" s="8" t="inlineStr">
         <is>
@@ -13449,7 +13457,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F201" s="8" t="inlineStr"/>
+      <c r="F201" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wellsfargo.com</t>
+        </is>
+      </c>
       <c r="G201" s="8" t="inlineStr"/>
       <c r="H201" s="8" t="inlineStr">
         <is>
@@ -13509,7 +13521,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F202" s="8" t="inlineStr"/>
+      <c r="F202" s="9" t="inlineStr">
+        <is>
+          <t>https://www.capitalone.com</t>
+        </is>
+      </c>
       <c r="G202" s="8" t="inlineStr"/>
       <c r="H202" s="8" t="inlineStr">
         <is>
@@ -13569,7 +13585,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F203" s="8" t="inlineStr"/>
+      <c r="F203" s="9" t="inlineStr">
+        <is>
+          <t>https://www.usbank.com</t>
+        </is>
+      </c>
       <c r="G203" s="8" t="inlineStr"/>
       <c r="H203" s="8" t="inlineStr">
         <is>
@@ -13629,7 +13649,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F204" s="8" t="inlineStr"/>
+      <c r="F204" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pnc.com</t>
+        </is>
+      </c>
       <c r="G204" s="8" t="inlineStr"/>
       <c r="H204" s="8" t="inlineStr">
         <is>
@@ -13689,7 +13713,11 @@
           <t>us</t>
         </is>
       </c>
-      <c r="F205" s="8" t="inlineStr"/>
+      <c r="F205" s="9" t="inlineStr">
+        <is>
+          <t>https://www.chime.com</t>
+        </is>
+      </c>
       <c r="G205" s="8" t="inlineStr"/>
       <c r="H205" s="8" t="inlineStr">
         <is>
@@ -13749,7 +13777,11 @@
           <t>gb</t>
         </is>
       </c>
-      <c r="F206" s="8" t="inlineStr"/>
+      <c r="F206" s="9" t="inlineStr">
+        <is>
+          <t>https://www.barclays.co.uk</t>
+        </is>
+      </c>
       <c r="G206" s="8" t="inlineStr"/>
       <c r="H206" s="8" t="inlineStr">
         <is>
@@ -13809,7 +13841,11 @@
           <t>gb</t>
         </is>
       </c>
-      <c r="F207" s="8" t="inlineStr"/>
+      <c r="F207" s="9" t="inlineStr">
+        <is>
+          <t>https://www.lloydsbank.com</t>
+        </is>
+      </c>
       <c r="G207" s="8" t="inlineStr"/>
       <c r="H207" s="8" t="inlineStr">
         <is>
@@ -13869,7 +13905,11 @@
           <t>gb</t>
         </is>
       </c>
-      <c r="F208" s="8" t="inlineStr"/>
+      <c r="F208" s="9" t="inlineStr">
+        <is>
+          <t>https://www.natwest.com</t>
+        </is>
+      </c>
       <c r="G208" s="8" t="inlineStr"/>
       <c r="H208" s="8" t="inlineStr">
         <is>
@@ -13929,7 +13969,11 @@
           <t>gb</t>
         </is>
       </c>
-      <c r="F209" s="8" t="inlineStr"/>
+      <c r="F209" s="9" t="inlineStr">
+        <is>
+          <t>https://www.santander.co.uk</t>
+        </is>
+      </c>
       <c r="G209" s="8" t="inlineStr"/>
       <c r="H209" s="8" t="inlineStr">
         <is>
@@ -13989,7 +14033,11 @@
           <t>gb</t>
         </is>
       </c>
-      <c r="F210" s="8" t="inlineStr"/>
+      <c r="F210" s="9" t="inlineStr">
+        <is>
+          <t>https://monzo.com</t>
+        </is>
+      </c>
       <c r="G210" s="8" t="inlineStr"/>
       <c r="H210" s="8" t="inlineStr">
         <is>
@@ -14049,7 +14097,11 @@
           <t>de</t>
         </is>
       </c>
-      <c r="F211" s="8" t="inlineStr"/>
+      <c r="F211" s="9" t="inlineStr">
+        <is>
+          <t>https://www.deutsche-bank.de</t>
+        </is>
+      </c>
       <c r="G211" s="8" t="inlineStr"/>
       <c r="H211" s="8" t="inlineStr">
         <is>
@@ -14109,7 +14161,11 @@
           <t>de</t>
         </is>
       </c>
-      <c r="F212" s="8" t="inlineStr"/>
+      <c r="F212" s="9" t="inlineStr">
+        <is>
+          <t>https://www.commerzbank.de</t>
+        </is>
+      </c>
       <c r="G212" s="8" t="inlineStr"/>
       <c r="H212" s="8" t="inlineStr">
         <is>
@@ -14169,7 +14225,11 @@
           <t>de</t>
         </is>
       </c>
-      <c r="F213" s="8" t="inlineStr"/>
+      <c r="F213" s="9" t="inlineStr">
+        <is>
+          <t>https://n26.com</t>
+        </is>
+      </c>
       <c r="G213" s="8" t="inlineStr"/>
       <c r="H213" s="8" t="inlineStr">
         <is>
@@ -14229,7 +14289,11 @@
           <t>fr</t>
         </is>
       </c>
-      <c r="F214" s="8" t="inlineStr"/>
+      <c r="F214" s="9" t="inlineStr">
+        <is>
+          <t>https://www.bnpparibas.com</t>
+        </is>
+      </c>
       <c r="G214" s="8" t="inlineStr"/>
       <c r="H214" s="8" t="inlineStr">
         <is>
@@ -14289,7 +14353,11 @@
           <t>fr</t>
         </is>
       </c>
-      <c r="F215" s="8" t="inlineStr"/>
+      <c r="F215" s="9" t="inlineStr">
+        <is>
+          <t>https://www.societegenerale.com</t>
+        </is>
+      </c>
       <c r="G215" s="8" t="inlineStr"/>
       <c r="H215" s="8" t="inlineStr">
         <is>
@@ -14349,7 +14417,11 @@
           <t>fr</t>
         </is>
       </c>
-      <c r="F216" s="8" t="inlineStr"/>
+      <c r="F216" s="9" t="inlineStr">
+        <is>
+          <t>https://www.credit-agricole.com</t>
+        </is>
+      </c>
       <c r="G216" s="8" t="inlineStr"/>
       <c r="H216" s="8" t="inlineStr">
         <is>
@@ -14409,7 +14481,11 @@
           <t>nl</t>
         </is>
       </c>
-      <c r="F217" s="8" t="inlineStr"/>
+      <c r="F217" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ing.nl</t>
+        </is>
+      </c>
       <c r="G217" s="8" t="inlineStr"/>
       <c r="H217" s="8" t="inlineStr">
         <is>
@@ -14469,7 +14545,11 @@
           <t>nl</t>
         </is>
       </c>
-      <c r="F218" s="8" t="inlineStr"/>
+      <c r="F218" s="9" t="inlineStr">
+        <is>
+          <t>https://www.abnamro.nl</t>
+        </is>
+      </c>
       <c r="G218" s="8" t="inlineStr"/>
       <c r="H218" s="8" t="inlineStr">
         <is>
@@ -14529,7 +14609,11 @@
           <t>nl</t>
         </is>
       </c>
-      <c r="F219" s="8" t="inlineStr"/>
+      <c r="F219" s="9" t="inlineStr">
+        <is>
+          <t>https://www.rabobank.nl</t>
+        </is>
+      </c>
       <c r="G219" s="8" t="inlineStr"/>
       <c r="H219" s="8" t="inlineStr">
         <is>
@@ -14589,7 +14673,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F220" s="8" t="inlineStr"/>
+      <c r="F220" s="9" t="inlineStr">
+        <is>
+          <t>https://www.boc.cn</t>
+        </is>
+      </c>
       <c r="G220" s="8" t="inlineStr"/>
       <c r="H220" s="8" t="inlineStr">
         <is>
@@ -14649,7 +14737,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F221" s="8" t="inlineStr"/>
+      <c r="F221" s="9" t="inlineStr">
+        <is>
+          <t>https://www.icbc.com.cn</t>
+        </is>
+      </c>
       <c r="G221" s="8" t="inlineStr"/>
       <c r="H221" s="8" t="inlineStr">
         <is>
@@ -14709,7 +14801,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F222" s="8" t="inlineStr"/>
+      <c r="F222" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ccb.com</t>
+        </is>
+      </c>
       <c r="G222" s="8" t="inlineStr"/>
       <c r="H222" s="8" t="inlineStr">
         <is>
@@ -14769,7 +14865,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F223" s="8" t="inlineStr"/>
+      <c r="F223" s="9" t="inlineStr">
+        <is>
+          <t>https://www.abchina.com</t>
+        </is>
+      </c>
       <c r="G223" s="8" t="inlineStr"/>
       <c r="H223" s="8" t="inlineStr">
         <is>
@@ -14829,7 +14929,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F224" s="8" t="inlineStr"/>
+      <c r="F224" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cmbchina.com</t>
+        </is>
+      </c>
       <c r="G224" s="8" t="inlineStr"/>
       <c r="H224" s="8" t="inlineStr">
         <is>
@@ -14889,7 +14993,11 @@
           <t>au</t>
         </is>
       </c>
-      <c r="F225" s="8" t="inlineStr"/>
+      <c r="F225" s="9" t="inlineStr">
+        <is>
+          <t>https://www.commbank.com.au</t>
+        </is>
+      </c>
       <c r="G225" s="8" t="inlineStr"/>
       <c r="H225" s="8" t="inlineStr">
         <is>
@@ -14949,7 +15057,11 @@
           <t>au</t>
         </is>
       </c>
-      <c r="F226" s="8" t="inlineStr"/>
+      <c r="F226" s="9" t="inlineStr">
+        <is>
+          <t>https://www.westpac.com.au</t>
+        </is>
+      </c>
       <c r="G226" s="8" t="inlineStr"/>
       <c r="H226" s="8" t="inlineStr">
         <is>
@@ -15009,7 +15121,11 @@
           <t>au</t>
         </is>
       </c>
-      <c r="F227" s="8" t="inlineStr"/>
+      <c r="F227" s="9" t="inlineStr">
+        <is>
+          <t>https://www.anz.com.au</t>
+        </is>
+      </c>
       <c r="G227" s="8" t="inlineStr"/>
       <c r="H227" s="8" t="inlineStr">
         <is>
@@ -15069,7 +15185,11 @@
           <t>au</t>
         </is>
       </c>
-      <c r="F228" s="8" t="inlineStr"/>
+      <c r="F228" s="9" t="inlineStr">
+        <is>
+          <t>https://www.nab.com.au</t>
+        </is>
+      </c>
       <c r="G228" s="8" t="inlineStr"/>
       <c r="H228" s="8" t="inlineStr">
         <is>
@@ -15129,7 +15249,11 @@
           <t>ca</t>
         </is>
       </c>
-      <c r="F229" s="8" t="inlineStr"/>
+      <c r="F229" s="9" t="inlineStr">
+        <is>
+          <t>https://www.rbc.com</t>
+        </is>
+      </c>
       <c r="G229" s="8" t="inlineStr"/>
       <c r="H229" s="8" t="inlineStr">
         <is>
@@ -15189,7 +15313,11 @@
           <t>ca</t>
         </is>
       </c>
-      <c r="F230" s="8" t="inlineStr"/>
+      <c r="F230" s="9" t="inlineStr">
+        <is>
+          <t>https://www.td.com</t>
+        </is>
+      </c>
       <c r="G230" s="8" t="inlineStr"/>
       <c r="H230" s="8" t="inlineStr">
         <is>
@@ -15249,7 +15377,11 @@
           <t>ca</t>
         </is>
       </c>
-      <c r="F231" s="8" t="inlineStr"/>
+      <c r="F231" s="9" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com</t>
+        </is>
+      </c>
       <c r="G231" s="8" t="inlineStr"/>
       <c r="H231" s="8" t="inlineStr">
         <is>
@@ -15309,7 +15441,11 @@
           <t>jp</t>
         </is>
       </c>
-      <c r="F232" s="8" t="inlineStr"/>
+      <c r="F232" s="9" t="inlineStr">
+        <is>
+          <t>https://www.bk.mufg.jp</t>
+        </is>
+      </c>
       <c r="G232" s="8" t="inlineStr"/>
       <c r="H232" s="8" t="inlineStr">
         <is>
@@ -15369,7 +15505,11 @@
           <t>jp</t>
         </is>
       </c>
-      <c r="F233" s="8" t="inlineStr"/>
+      <c r="F233" s="9" t="inlineStr">
+        <is>
+          <t>https://www.smbc.co.jp</t>
+        </is>
+      </c>
       <c r="G233" s="8" t="inlineStr"/>
       <c r="H233" s="8" t="inlineStr">
         <is>
@@ -15429,7 +15569,11 @@
           <t>jp</t>
         </is>
       </c>
-      <c r="F234" s="8" t="inlineStr"/>
+      <c r="F234" s="9" t="inlineStr">
+        <is>
+          <t>https://www.jp-bank.japanpost.jp</t>
+        </is>
+      </c>
       <c r="G234" s="8" t="inlineStr"/>
       <c r="H234" s="8" t="inlineStr">
         <is>
@@ -15489,7 +15633,11 @@
           <t>kr</t>
         </is>
       </c>
-      <c r="F235" s="8" t="inlineStr"/>
+      <c r="F235" s="9" t="inlineStr">
+        <is>
+          <t>https://www.kbstar.com</t>
+        </is>
+      </c>
       <c r="G235" s="8" t="inlineStr"/>
       <c r="H235" s="8" t="inlineStr">
         <is>
@@ -15549,7 +15697,11 @@
           <t>kr</t>
         </is>
       </c>
-      <c r="F236" s="8" t="inlineStr"/>
+      <c r="F236" s="9" t="inlineStr">
+        <is>
+          <t>https://www.shinhan.com</t>
+        </is>
+      </c>
       <c r="G236" s="8" t="inlineStr"/>
       <c r="H236" s="8" t="inlineStr">
         <is>
@@ -15609,7 +15761,11 @@
           <t>kr</t>
         </is>
       </c>
-      <c r="F237" s="8" t="inlineStr"/>
+      <c r="F237" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wooribank.com</t>
+        </is>
+      </c>
       <c r="G237" s="8" t="inlineStr"/>
       <c r="H237" s="8" t="inlineStr">
         <is>
@@ -15669,7 +15825,11 @@
           <t>hk</t>
         </is>
       </c>
-      <c r="F238" s="8" t="inlineStr"/>
+      <c r="F238" s="9" t="inlineStr">
+        <is>
+          <t>https://www.hangseng.com</t>
+        </is>
+      </c>
       <c r="G238" s="8" t="inlineStr"/>
       <c r="H238" s="8" t="inlineStr">
         <is>
@@ -15729,7 +15889,11 @@
           <t>hk</t>
         </is>
       </c>
-      <c r="F239" s="8" t="inlineStr"/>
+      <c r="F239" s="9" t="inlineStr">
+        <is>
+          <t>https://www.bochk.com</t>
+        </is>
+      </c>
       <c r="G239" s="8" t="inlineStr"/>
       <c r="H239" s="8" t="inlineStr">
         <is>
@@ -16269,7 +16433,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F248" s="8" t="inlineStr"/>
+      <c r="F248" s="9" t="inlineStr">
+        <is>
+          <t>https://www.alipay.com</t>
+        </is>
+      </c>
       <c r="G248" s="8" t="inlineStr"/>
       <c r="H248" s="8" t="inlineStr">
         <is>
@@ -16329,7 +16497,11 @@
           <t>cn</t>
         </is>
       </c>
-      <c r="F249" s="8" t="inlineStr"/>
+      <c r="F249" s="9" t="inlineStr">
+        <is>
+          <t>https://pay.weixin.qq.com</t>
+        </is>
+      </c>
       <c r="G249" s="8" t="inlineStr"/>
       <c r="H249" s="8" t="inlineStr">
         <is>
@@ -16389,7 +16561,11 @@
           <t>gb</t>
         </is>
       </c>
-      <c r="F250" s="8" t="inlineStr"/>
+      <c r="F250" s="9" t="inlineStr">
+        <is>
+          <t>https://www.revolut.com</t>
+        </is>
+      </c>
       <c r="G250" s="8" t="inlineStr"/>
       <c r="H250" s="8" t="inlineStr">
         <is>
@@ -16607,14 +16783,58 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F240" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F241" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F242" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F208" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F214" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F215" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F216" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F217" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F218" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F219" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F220" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F221" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F222" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F223" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F224" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F225" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F226" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F227" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F228" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F229" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F230" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F231" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F232" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F233" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F234" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F235" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F236" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F237" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F238" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F239" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F240" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F241" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F242" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId233"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>